<commit_message>
Changes to be committed: 	modified:   Admin/Course Attendance.xlsx 	renamed:    Stage1-C++-Beginner/2790-Knowing Variables/2790-Knowing Variables.pptx -> Stage1-C++-Beginner/2790-Know the Variables/2790-Know the Variables.pptx 	renamed:    Stage1-C++-Beginner/2790-Knowing Variables/cast -> Stage1-C++-Beginner/2790-Know the Variables/cast 	renamed:    Stage1-C++-Beginner/2790-Knowing Variables/cast.cpp -> Stage1-C++-Beginner/2790-Know the Variables/cast.cpp 	modified:   Stage1-C++-Beginner/2791-Branching 1.pptx 	new file:   Stage1-C++-Beginner/2791-Branching 1/2791-Branching 1.pptx 	modified:   Stage3-Informatics-Elementary-B/Trees/Elementary B - Trees.pptx
</commit_message>
<xml_diff>
--- a/Admin/Course Attendance.xlsx
+++ b/Admin/Course Attendance.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/851caa7714272873/CLASSES-Informatics/Admin/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="480" documentId="13_ncr:1_{10AACCFA-37B1-6D44-A367-828EAD02C19B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F237102B-B8AE-2146-A24A-5A2588C80088}"/>
+  <xr:revisionPtr revIDLastSave="527" documentId="13_ncr:1_{10AACCFA-37B1-6D44-A367-828EAD02C19B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2C59B26C-DB70-4287-9D08-3A9620C2AC17}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="25740" windowHeight="15720" activeTab="1" xr2:uid="{24CAAD2F-8633-184E-A7D2-D706FBAD8E49}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11520" activeTab="3" xr2:uid="{24CAAD2F-8633-184E-A7D2-D706FBAD8E49}"/>
   </bookViews>
   <sheets>
     <sheet name="Student Information" sheetId="3" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="166">
   <si>
     <t>Class 1</t>
   </si>
@@ -498,6 +498,45 @@
   </si>
   <si>
     <t>Class 13</t>
+  </si>
+  <si>
+    <t>Shaurya Thakur</t>
+  </si>
+  <si>
+    <t>Hornsby North Public School</t>
+  </si>
+  <si>
+    <t>Aiden Wang</t>
+  </si>
+  <si>
+    <t>lyr8322@gmail.com</t>
+  </si>
+  <si>
+    <t>Samuel Gilbert Public School</t>
+  </si>
+  <si>
+    <t>Sean Mok</t>
+  </si>
+  <si>
+    <t>sean.mok484@education.nsw.gov.au</t>
+  </si>
+  <si>
+    <t>Baulkham Hills North Public School</t>
+  </si>
+  <si>
+    <t>Class 14</t>
+  </si>
+  <si>
+    <t>Simulation and Binary Trees</t>
+  </si>
+  <si>
+    <t>Simulation with 2022 problems, Binary tree representation, complete binary trees, binary tree traversal</t>
+  </si>
+  <si>
+    <t>First Encounter, Know the Variables</t>
+  </si>
+  <si>
+    <t>Know the Variables, review homework</t>
   </si>
 </sst>
 </file>
@@ -546,6 +585,7 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -974,15 +1014,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91FB8569-CA3E-974B-8804-A3AC313A4BC3}">
-  <dimension ref="A1:E21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:E24"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.9" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="3" max="3" width="33.83203125" customWidth="1"/>
-    <col min="4" max="4" width="36.83203125" customWidth="1"/>
+    <col min="3" max="3" width="33.85546875" customWidth="1"/>
+    <col min="4" max="4" width="36.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>19</v>
       </c>
@@ -999,7 +1039,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -1016,7 +1056,7 @@
         <v>2025</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
@@ -1033,7 +1073,7 @@
         <v>2025</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
@@ -1050,7 +1090,7 @@
         <v>2025</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>16</v>
       </c>
@@ -1067,7 +1107,7 @@
         <v>2025</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>85</v>
       </c>
@@ -1084,7 +1124,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>90</v>
       </c>
@@ -1101,7 +1141,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>91</v>
       </c>
@@ -1118,7 +1158,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
         <v>110</v>
       </c>
@@ -1135,7 +1175,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
         <v>87</v>
       </c>
@@ -1152,7 +1192,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A11" s="1" t="s">
         <v>95</v>
       </c>
@@ -1169,7 +1209,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A12" s="1" t="s">
         <v>115</v>
       </c>
@@ -1186,7 +1226,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
         <v>102</v>
       </c>
@@ -1203,7 +1243,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A14" s="1" t="s">
         <v>106</v>
       </c>
@@ -1220,7 +1260,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
         <v>130</v>
       </c>
@@ -1237,7 +1277,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A16" s="1" t="s">
         <v>131</v>
       </c>
@@ -1254,7 +1294,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A17" s="1" t="s">
         <v>132</v>
       </c>
@@ -1271,7 +1311,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A18" s="1" t="s">
         <v>135</v>
       </c>
@@ -1288,7 +1328,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A19" s="1" t="s">
         <v>133</v>
       </c>
@@ -1305,7 +1345,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A20" s="1" t="s">
         <v>136</v>
       </c>
@@ -1322,7 +1362,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A21" s="1" t="s">
         <v>150</v>
       </c>
@@ -1337,6 +1377,51 @@
       </c>
       <c r="E21">
         <v>2026</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A22" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="B22">
+        <v>6</v>
+      </c>
+      <c r="C22" t="s">
+        <v>154</v>
+      </c>
+      <c r="E22">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A23" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="B23">
+        <v>5</v>
+      </c>
+      <c r="C23" t="s">
+        <v>157</v>
+      </c>
+      <c r="D23" s="16" t="s">
+        <v>156</v>
+      </c>
+      <c r="E23">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A24" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="B24">
+        <v>6</v>
+      </c>
+      <c r="C24" t="s">
+        <v>160</v>
+      </c>
+      <c r="D24" t="s">
+        <v>159</v>
       </c>
     </row>
   </sheetData>
@@ -1369,17 +1454,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05115B71-C326-1145-853C-2345070572D9}">
   <dimension ref="A1:P28"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="12.9" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="9.1640625" style="4" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" style="4" customWidth="1"/>
     <col min="2" max="2" width="13.5" style="4" customWidth="1"/>
-    <col min="3" max="3" width="13.33203125" style="3" customWidth="1"/>
-    <col min="4" max="8" width="3.83203125" style="3" customWidth="1"/>
-    <col min="9" max="14" width="15.83203125" style="3" customWidth="1"/>
-    <col min="15" max="16384" width="10.83203125" style="4"/>
+    <col min="3" max="3" width="13.35546875" style="3" customWidth="1"/>
+    <col min="4" max="8" width="3.85546875" style="3" customWidth="1"/>
+    <col min="9" max="14" width="15.85546875" style="3" customWidth="1"/>
+    <col min="15" max="16384" width="10.85546875" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="15" customFormat="1" ht="32" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" s="15" customFormat="1" ht="31.75" x14ac:dyDescent="0.45">
       <c r="A1" s="13" t="s">
         <v>5</v>
       </c>
@@ -1397,7 +1482,7 @@
       <c r="M1" s="14"/>
       <c r="N1" s="14"/>
     </row>
-    <row r="2" spans="1:16" ht="80" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:16" ht="80.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="9" t="s">
         <v>1</v>
       </c>
@@ -1437,7 +1522,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A3" s="5" t="s">
         <v>0</v>
       </c>
@@ -1479,7 +1564,7 @@
       </c>
       <c r="P3" s="8"/>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A4" s="5" t="s">
         <v>12</v>
       </c>
@@ -1508,7 +1593,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A5" s="5" t="s">
         <v>0</v>
       </c>
@@ -1547,7 +1632,7 @@
       </c>
       <c r="P5" s="8"/>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A6" s="5" t="s">
         <v>26</v>
       </c>
@@ -1574,7 +1659,7 @@
       <c r="O6" s="8"/>
       <c r="P6" s="8"/>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A7" s="5" t="s">
         <v>12</v>
       </c>
@@ -1607,7 +1692,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A8" s="5" t="s">
         <v>28</v>
       </c>
@@ -1638,7 +1723,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A9" s="5" t="s">
         <v>26</v>
       </c>
@@ -1671,7 +1756,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A10" s="5" t="s">
         <v>29</v>
       </c>
@@ -1702,7 +1787,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A11" s="5" t="s">
         <v>28</v>
       </c>
@@ -1735,7 +1820,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A12" s="5" t="s">
         <v>31</v>
       </c>
@@ -1768,7 +1853,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A13" s="5" t="s">
         <v>33</v>
       </c>
@@ -1792,7 +1877,7 @@
       <c r="O13" s="8"/>
       <c r="P13" s="8"/>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A14" s="5" t="s">
         <v>34</v>
       </c>
@@ -1831,7 +1916,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A15" s="5" t="s">
         <v>79</v>
       </c>
@@ -1854,7 +1939,7 @@
       <c r="N15" s="8"/>
       <c r="O15" s="8"/>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A16" s="5" t="s">
         <v>0</v>
       </c>
@@ -1888,7 +1973,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A17" s="5" t="s">
         <v>12</v>
       </c>
@@ -1917,7 +2002,7 @@
       <c r="O17" s="8"/>
       <c r="P17" s="8"/>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A18" s="5" t="s">
         <v>26</v>
       </c>
@@ -1946,7 +2031,7 @@
       <c r="O18" s="8"/>
       <c r="P18" s="8"/>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A19" s="5" t="s">
         <v>28</v>
       </c>
@@ -1975,7 +2060,7 @@
       <c r="N19" s="8"/>
       <c r="O19" s="8"/>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A20" s="5" t="s">
         <v>29</v>
       </c>
@@ -2003,7 +2088,7 @@
       <c r="N20" s="8"/>
       <c r="O20" s="8"/>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A21" s="5" t="s">
         <v>31</v>
       </c>
@@ -2034,7 +2119,7 @@
       <c r="N21" s="8"/>
       <c r="O21" s="8"/>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A22" s="5" t="s">
         <v>34</v>
       </c>
@@ -2065,7 +2150,7 @@
       <c r="N22" s="8"/>
       <c r="O22" s="8"/>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A23" s="5"/>
       <c r="B23" s="6"/>
       <c r="C23" s="7"/>
@@ -2077,7 +2162,7 @@
       <c r="N23" s="8"/>
       <c r="O23" s="8"/>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A24" s="5"/>
       <c r="B24" s="6"/>
       <c r="C24" s="7"/>
@@ -2089,7 +2174,7 @@
       <c r="N24" s="8"/>
       <c r="O24" s="8"/>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A25" s="5"/>
       <c r="B25" s="6"/>
       <c r="C25" s="7"/>
@@ -2101,7 +2186,7 @@
       <c r="N25" s="8"/>
       <c r="O25" s="8"/>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A26" s="5"/>
       <c r="B26" s="6"/>
       <c r="C26" s="7"/>
@@ -2113,7 +2198,7 @@
       <c r="N26" s="8"/>
       <c r="O26" s="8"/>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A27" s="5"/>
       <c r="B27" s="6"/>
       <c r="C27" s="7"/>
@@ -2125,7 +2210,7 @@
       <c r="N27" s="8"/>
       <c r="O27" s="8"/>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A28" s="5"/>
       <c r="B28" s="6"/>
       <c r="C28" s="7"/>
@@ -2146,17 +2231,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1940DD8-A835-C84C-9FD6-C7272FA36228}">
   <dimension ref="A1:O28"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="12.9" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="9.1640625" style="4" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" style="4" customWidth="1"/>
     <col min="2" max="2" width="13.5" style="4" customWidth="1"/>
-    <col min="3" max="3" width="13.33203125" style="3" customWidth="1"/>
-    <col min="4" max="7" width="3.83203125" style="3" customWidth="1"/>
-    <col min="8" max="13" width="15.83203125" style="3" customWidth="1"/>
-    <col min="14" max="16384" width="10.83203125" style="4"/>
+    <col min="3" max="3" width="13.35546875" style="3" customWidth="1"/>
+    <col min="4" max="7" width="3.85546875" style="3" customWidth="1"/>
+    <col min="8" max="13" width="15.85546875" style="3" customWidth="1"/>
+    <col min="14" max="16384" width="10.85546875" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="15" customFormat="1" ht="32" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" s="15" customFormat="1" ht="31.75" x14ac:dyDescent="0.45">
       <c r="A1" s="13" t="s">
         <v>89</v>
       </c>
@@ -2173,7 +2258,7 @@
       <c r="L1" s="14"/>
       <c r="M1" s="14"/>
     </row>
-    <row r="2" spans="1:15" ht="80" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:15" ht="80.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="9" t="s">
         <v>1</v>
       </c>
@@ -2210,7 +2295,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A3" s="5" t="s">
         <v>0</v>
       </c>
@@ -2242,7 +2327,7 @@
       <c r="N3" s="8"/>
       <c r="O3" s="8"/>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A4" s="5" t="s">
         <v>12</v>
       </c>
@@ -2274,7 +2359,7 @@
       <c r="N4" s="8"/>
       <c r="O4" s="8"/>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A5" s="5" t="s">
         <v>26</v>
       </c>
@@ -2301,7 +2386,7 @@
       <c r="N5" s="8"/>
       <c r="O5" s="8"/>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A6" s="5" t="s">
         <v>28</v>
       </c>
@@ -2328,7 +2413,7 @@
       <c r="N6" s="8"/>
       <c r="O6" s="8"/>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A7" s="5" t="s">
         <v>29</v>
       </c>
@@ -2358,7 +2443,7 @@
       <c r="N7" s="8"/>
       <c r="O7" s="8"/>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A8" s="5" t="s">
         <v>31</v>
       </c>
@@ -2388,7 +2473,7 @@
       <c r="N8" s="8"/>
       <c r="O8" s="8"/>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A9" s="5" t="s">
         <v>34</v>
       </c>
@@ -2418,7 +2503,7 @@
       <c r="N9" s="8"/>
       <c r="O9" s="8"/>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A10" s="5" t="s">
         <v>122</v>
       </c>
@@ -2450,7 +2535,7 @@
       <c r="N10" s="8"/>
       <c r="O10" s="8"/>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A11" s="5" t="s">
         <v>123</v>
       </c>
@@ -2482,7 +2567,7 @@
       <c r="N11" s="8"/>
       <c r="O11" s="8"/>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A12" s="5" t="s">
         <v>124</v>
       </c>
@@ -2507,7 +2592,7 @@
       <c r="N12" s="8"/>
       <c r="O12" s="8"/>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A13" s="5" t="s">
         <v>125</v>
       </c>
@@ -2535,7 +2620,7 @@
       <c r="N13" s="8"/>
       <c r="O13" s="8"/>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A14" s="5" t="s">
         <v>126</v>
       </c>
@@ -2563,7 +2648,7 @@
       <c r="N14" s="8"/>
       <c r="O14" s="8"/>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A15" s="5" t="s">
         <v>152</v>
       </c>
@@ -2590,12 +2675,28 @@
       <c r="M15" s="8"/>
       <c r="N15" s="8"/>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A16" s="5"/>
-      <c r="B16" s="6"/>
-      <c r="C16" s="7"/>
-      <c r="H16" s="8"/>
-      <c r="I16" s="8"/>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.45">
+      <c r="A16" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="B16" s="6">
+        <v>46243</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="H16" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="I16" s="8" t="s">
+        <v>163</v>
+      </c>
       <c r="J16" s="8"/>
       <c r="K16" s="8"/>
       <c r="L16" s="8"/>
@@ -2603,7 +2704,7 @@
       <c r="N16" s="8"/>
       <c r="O16" s="8"/>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A17" s="5"/>
       <c r="B17" s="6"/>
       <c r="C17" s="7"/>
@@ -2616,7 +2717,7 @@
       <c r="N17" s="8"/>
       <c r="O17" s="8"/>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A18" s="5"/>
       <c r="B18" s="6"/>
       <c r="C18" s="7"/>
@@ -2629,7 +2730,7 @@
       <c r="N18" s="8"/>
       <c r="O18" s="8"/>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A19" s="5"/>
       <c r="B19" s="6"/>
       <c r="C19" s="7"/>
@@ -2641,7 +2742,7 @@
       <c r="M19" s="8"/>
       <c r="N19" s="8"/>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A20" s="5"/>
       <c r="B20" s="6"/>
       <c r="C20" s="7"/>
@@ -2653,7 +2754,7 @@
       <c r="M20" s="8"/>
       <c r="N20" s="8"/>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A21" s="5"/>
       <c r="B21" s="6"/>
       <c r="C21" s="7"/>
@@ -2665,7 +2766,7 @@
       <c r="M21" s="8"/>
       <c r="N21" s="8"/>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A22" s="5"/>
       <c r="B22" s="6"/>
       <c r="C22" s="7"/>
@@ -2677,7 +2778,7 @@
       <c r="M22" s="8"/>
       <c r="N22" s="8"/>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A23" s="5"/>
       <c r="B23" s="6"/>
       <c r="C23" s="7"/>
@@ -2689,7 +2790,7 @@
       <c r="M23" s="8"/>
       <c r="N23" s="8"/>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A24" s="5"/>
       <c r="B24" s="6"/>
       <c r="C24" s="7"/>
@@ -2701,7 +2802,7 @@
       <c r="M24" s="8"/>
       <c r="N24" s="8"/>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A25" s="5"/>
       <c r="B25" s="6"/>
       <c r="C25" s="7"/>
@@ -2713,7 +2814,7 @@
       <c r="M25" s="8"/>
       <c r="N25" s="8"/>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A26" s="5"/>
       <c r="B26" s="6"/>
       <c r="C26" s="7"/>
@@ -2725,7 +2826,7 @@
       <c r="M26" s="8"/>
       <c r="N26" s="8"/>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A27" s="5"/>
       <c r="B27" s="6"/>
       <c r="C27" s="7"/>
@@ -2737,7 +2838,7 @@
       <c r="M27" s="8"/>
       <c r="N27" s="8"/>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A28" s="5"/>
       <c r="B28" s="6"/>
       <c r="C28" s="7"/>
@@ -2758,17 +2859,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DFCB767-1FBD-9647-82C4-2908A24D9134}">
   <dimension ref="A1:T28"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="12.9" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="9.1640625" style="4" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" style="4" customWidth="1"/>
     <col min="2" max="2" width="13.5" style="4" customWidth="1"/>
-    <col min="3" max="3" width="13.33203125" style="3" customWidth="1"/>
-    <col min="4" max="12" width="3.83203125" style="3" customWidth="1"/>
-    <col min="13" max="18" width="15.83203125" style="3" customWidth="1"/>
-    <col min="19" max="16384" width="10.83203125" style="4"/>
+    <col min="3" max="3" width="13.35546875" style="3" customWidth="1"/>
+    <col min="4" max="14" width="3.85546875" style="3" customWidth="1"/>
+    <col min="15" max="18" width="15.85546875" style="3" customWidth="1"/>
+    <col min="19" max="16384" width="10.85546875" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" s="15" customFormat="1" ht="32" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:20" s="15" customFormat="1" ht="31.75" x14ac:dyDescent="0.45">
       <c r="A1" s="13" t="s">
         <v>94</v>
       </c>
@@ -2790,7 +2891,7 @@
       <c r="Q1" s="14"/>
       <c r="R1" s="14"/>
     </row>
-    <row r="2" spans="1:20" ht="80" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:20" ht="80.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="9" t="s">
         <v>1</v>
       </c>
@@ -2827,11 +2928,11 @@
       <c r="L2" s="10" t="s">
         <v>150</v>
       </c>
-      <c r="M2" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="N2" s="11" t="s">
-        <v>36</v>
+      <c r="M2" s="10" t="s">
+        <v>155</v>
+      </c>
+      <c r="N2" s="10" t="s">
+        <v>158</v>
       </c>
       <c r="O2" s="11"/>
       <c r="P2" s="11"/>
@@ -2842,7 +2943,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A3" s="5" t="s">
         <v>0</v>
       </c>
@@ -2879,20 +2980,18 @@
       <c r="L3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="M3" s="8" t="s">
+      <c r="O3" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="N3" s="8"/>
-      <c r="O3" s="8"/>
       <c r="P3" s="8"/>
       <c r="Q3" s="8"/>
       <c r="R3" s="8"/>
       <c r="S3" s="8"/>
       <c r="T3" s="8"/>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A4" s="5" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="B4" s="6">
         <v>46236</v>
@@ -2924,34 +3023,68 @@
       <c r="L4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="M4" s="8"/>
-      <c r="N4" s="8"/>
-      <c r="O4" s="8"/>
+      <c r="O4" s="8" t="s">
+        <v>164</v>
+      </c>
       <c r="P4" s="8"/>
       <c r="Q4" s="8"/>
       <c r="R4" s="8"/>
       <c r="S4" s="8"/>
       <c r="T4" s="8"/>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A5" s="5"/>
-      <c r="B5" s="6"/>
-      <c r="C5" s="7"/>
-      <c r="M5" s="8"/>
-      <c r="N5" s="8"/>
-      <c r="O5" s="8"/>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="A5" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="6">
+        <v>46243</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="M5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="N5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="O5" s="8" t="s">
+        <v>165</v>
+      </c>
       <c r="P5" s="8"/>
       <c r="Q5" s="8"/>
       <c r="R5" s="8"/>
       <c r="S5" s="8"/>
       <c r="T5" s="8"/>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A6" s="5"/>
       <c r="B6" s="6"/>
       <c r="C6" s="7"/>
-      <c r="M6" s="8"/>
-      <c r="N6" s="8"/>
       <c r="O6" s="8"/>
       <c r="P6" s="8"/>
       <c r="Q6" s="8"/>
@@ -2959,12 +3092,10 @@
       <c r="S6" s="8"/>
       <c r="T6" s="8"/>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A7" s="5"/>
       <c r="B7" s="6"/>
       <c r="C7" s="7"/>
-      <c r="M7" s="8"/>
-      <c r="N7" s="8"/>
       <c r="O7" s="8"/>
       <c r="P7" s="8"/>
       <c r="Q7" s="8"/>
@@ -2972,12 +3103,10 @@
       <c r="S7" s="8"/>
       <c r="T7" s="8"/>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A8" s="5"/>
       <c r="B8" s="6"/>
       <c r="C8" s="7"/>
-      <c r="M8" s="8"/>
-      <c r="N8" s="8"/>
       <c r="O8" s="8"/>
       <c r="P8" s="8"/>
       <c r="Q8" s="8"/>
@@ -2985,12 +3114,10 @@
       <c r="S8" s="8"/>
       <c r="T8" s="8"/>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A9" s="5"/>
       <c r="B9" s="6"/>
       <c r="C9" s="7"/>
-      <c r="M9" s="8"/>
-      <c r="N9" s="8"/>
       <c r="O9" s="8"/>
       <c r="P9" s="8"/>
       <c r="Q9" s="8"/>
@@ -2998,12 +3125,10 @@
       <c r="S9" s="8"/>
       <c r="T9" s="8"/>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A10" s="5"/>
       <c r="B10" s="6"/>
       <c r="C10" s="7"/>
-      <c r="M10" s="8"/>
-      <c r="N10" s="8"/>
       <c r="O10" s="8"/>
       <c r="P10" s="8"/>
       <c r="Q10" s="8"/>
@@ -3011,12 +3136,10 @@
       <c r="S10" s="8"/>
       <c r="T10" s="8"/>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A11" s="5"/>
       <c r="B11" s="6"/>
       <c r="C11" s="7"/>
-      <c r="M11" s="8"/>
-      <c r="N11" s="8"/>
       <c r="O11" s="8"/>
       <c r="P11" s="8"/>
       <c r="Q11" s="8"/>
@@ -3024,12 +3147,10 @@
       <c r="S11" s="8"/>
       <c r="T11" s="8"/>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A12" s="5"/>
       <c r="B12" s="6"/>
       <c r="C12" s="7"/>
-      <c r="M12" s="8"/>
-      <c r="N12" s="8"/>
       <c r="O12" s="8"/>
       <c r="P12" s="8"/>
       <c r="Q12" s="8"/>
@@ -3037,12 +3158,10 @@
       <c r="S12" s="8"/>
       <c r="T12" s="8"/>
     </row>
-    <row r="13" spans="1:20" ht="16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:20" ht="15.9" x14ac:dyDescent="0.45">
       <c r="A13" s="5"/>
       <c r="B13" s="6"/>
       <c r="C13" s="7"/>
-      <c r="M13" s="8"/>
-      <c r="N13" s="1"/>
       <c r="O13" s="1"/>
       <c r="P13" s="1"/>
       <c r="Q13" s="1"/>
@@ -3050,11 +3169,10 @@
       <c r="S13" s="1"/>
       <c r="T13" s="8"/>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A14" s="5"/>
       <c r="B14" s="6"/>
       <c r="C14" s="7"/>
-      <c r="M14" s="8"/>
       <c r="O14" s="8"/>
       <c r="P14" s="8"/>
       <c r="Q14" s="8"/>
@@ -3062,22 +3180,20 @@
       <c r="S14" s="8"/>
       <c r="T14" s="8"/>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A15" s="5"/>
       <c r="B15" s="6"/>
       <c r="C15" s="7"/>
-      <c r="M15" s="8"/>
       <c r="O15" s="8"/>
       <c r="P15" s="8"/>
       <c r="Q15" s="8"/>
       <c r="R15" s="8"/>
       <c r="S15" s="8"/>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A16" s="5"/>
       <c r="B16" s="6"/>
       <c r="C16" s="7"/>
-      <c r="M16" s="8"/>
       <c r="O16" s="8"/>
       <c r="P16" s="8"/>
       <c r="Q16" s="8"/>
@@ -3085,11 +3201,10 @@
       <c r="S16" s="8"/>
       <c r="T16" s="8"/>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A17" s="5"/>
       <c r="B17" s="6"/>
       <c r="C17" s="7"/>
-      <c r="M17" s="8"/>
       <c r="O17" s="8"/>
       <c r="P17" s="8"/>
       <c r="Q17" s="8"/>
@@ -3097,11 +3212,10 @@
       <c r="S17" s="8"/>
       <c r="T17" s="8"/>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A18" s="5"/>
       <c r="B18" s="6"/>
       <c r="C18" s="7"/>
-      <c r="M18" s="8"/>
       <c r="O18" s="8"/>
       <c r="P18" s="8"/>
       <c r="Q18" s="8"/>
@@ -3109,120 +3223,100 @@
       <c r="S18" s="8"/>
       <c r="T18" s="8"/>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A19" s="5"/>
       <c r="B19" s="6"/>
       <c r="C19" s="7"/>
-      <c r="M19" s="8"/>
-      <c r="N19" s="8"/>
       <c r="O19" s="8"/>
       <c r="P19" s="8"/>
       <c r="Q19" s="8"/>
       <c r="R19" s="8"/>
       <c r="S19" s="8"/>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A20" s="5"/>
       <c r="B20" s="6"/>
       <c r="C20" s="7"/>
-      <c r="M20" s="8"/>
-      <c r="N20" s="8"/>
       <c r="O20" s="8"/>
       <c r="P20" s="8"/>
       <c r="Q20" s="8"/>
       <c r="R20" s="8"/>
       <c r="S20" s="8"/>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A21" s="5"/>
       <c r="B21" s="6"/>
       <c r="C21" s="7"/>
-      <c r="M21" s="8"/>
-      <c r="N21" s="8"/>
       <c r="O21" s="8"/>
       <c r="P21" s="8"/>
       <c r="Q21" s="8"/>
       <c r="R21" s="8"/>
       <c r="S21" s="8"/>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A22" s="5"/>
       <c r="B22" s="6"/>
       <c r="C22" s="7"/>
-      <c r="M22" s="8"/>
-      <c r="N22" s="8"/>
       <c r="O22" s="8"/>
       <c r="P22" s="8"/>
       <c r="Q22" s="8"/>
       <c r="R22" s="8"/>
       <c r="S22" s="8"/>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A23" s="5"/>
       <c r="B23" s="6"/>
       <c r="C23" s="7"/>
-      <c r="M23" s="8"/>
-      <c r="N23" s="8"/>
       <c r="O23" s="8"/>
       <c r="P23" s="8"/>
       <c r="Q23" s="8"/>
       <c r="R23" s="8"/>
       <c r="S23" s="8"/>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A24" s="5"/>
       <c r="B24" s="6"/>
       <c r="C24" s="7"/>
-      <c r="M24" s="8"/>
-      <c r="N24" s="8"/>
       <c r="O24" s="8"/>
       <c r="P24" s="8"/>
       <c r="Q24" s="8"/>
       <c r="R24" s="8"/>
       <c r="S24" s="8"/>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A25" s="5"/>
       <c r="B25" s="6"/>
       <c r="C25" s="7"/>
-      <c r="M25" s="8"/>
-      <c r="N25" s="8"/>
       <c r="O25" s="8"/>
       <c r="P25" s="8"/>
       <c r="Q25" s="8"/>
       <c r="R25" s="8"/>
       <c r="S25" s="8"/>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A26" s="5"/>
       <c r="B26" s="6"/>
       <c r="C26" s="7"/>
-      <c r="M26" s="8"/>
-      <c r="N26" s="8"/>
       <c r="O26" s="8"/>
       <c r="P26" s="8"/>
       <c r="Q26" s="8"/>
       <c r="R26" s="8"/>
       <c r="S26" s="8"/>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A27" s="5"/>
       <c r="B27" s="6"/>
       <c r="C27" s="7"/>
-      <c r="M27" s="8"/>
-      <c r="N27" s="8"/>
       <c r="O27" s="8"/>
       <c r="P27" s="8"/>
       <c r="Q27" s="8"/>
       <c r="R27" s="8"/>
       <c r="S27" s="8"/>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A28" s="5"/>
       <c r="B28" s="6"/>
       <c r="C28" s="7"/>
-      <c r="M28" s="8"/>
-      <c r="N28" s="8"/>
       <c r="O28" s="8"/>
       <c r="P28" s="8"/>
       <c r="Q28" s="8"/>

</xml_diff>